<commit_message>
EAINT-12341: cover every Pre-Application business type
- CH7 Business Trading (Sarawak) next to CH5 (Sabah); the robot picks the
  Sarawak radio and reads a trading run's TIN from tab "1 Companies".
- CH8 Sdn Bhd / Bhd, 4 Malaysian directors (QA request) next to CH3
  (foreign director); new TS08A, TS15/TS19 extended.
- Workbook, scenarios.yaml, eSim setup sheet, npm scripts, guide and
  status updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015cZiRisoA6SpsRKpMC9zuJ
</commit_message>
<xml_diff>
--- a/EAINT-12341/cr/EAINT-12341/02-plan/EAINT-12341_Test_Case_v1.3.xlsx
+++ b/EAINT-12341/cr/EAINT-12341/02-plan/EAINT-12341_Test_Case_v1.3.xlsx
@@ -495,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O44"/>
+  <dimension ref="A1:O45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1363,124 +1363,124 @@
     <row r="24" ht="92" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
         <is>
+          <t>12341_TS08A</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Sdn Bhd / Bhd</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>4 directors</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>All Malaysian</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Email Template 1 (combined)</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Precondition: chain 12341_CH8 has been executed by the automation up to Application Approved (see the 'Test Data &amp; Chains' sheet). The run log's READY FOR MANUAL EMAIL CHECK block gives the UCD email, Application No, Pre-Application No, company name, BRNs and the approval timestamp used below.
+1. In Mailtrap, search for chain CH8's UCD email.
+2. Open the guideline email; check To/CC, subject and body against TS01–TS03 and TS05.</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Ensure:
+• Combined Email Template 1 received with CH8's values; To = UCD email, CC = apply@eauto.my, Appointment Letter attached.</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Sdn Bhd, 4 directors, all Malaysian → the same combined guideline email
+Added 02.10.2026 at the QA's request: Sdn Bhd / Bhd covered by a normal case as well as the foreign-director case (TS08).</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>12341_CH8</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>REQ-005 (Example 1)</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>Functional / Positive</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr"/>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25" ht="92" customHeight="1">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
           <t>12341_TS09</t>
         </is>
       </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="B25" s="2" t="inlineStr">
         <is>
           <t>LLP</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
+      <c r="C25" s="2" t="inlineStr">
         <is>
           <t>4 partners</t>
         </is>
       </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>All Malaysian</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>Email Template 1 (combined)</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="F25" s="2" t="inlineStr">
         <is>
           <t>Precondition: chain 12341_CH4 has been executed by the automation up to Application Approved (see the 'Test Data &amp; Chains' sheet). The run log's READY FOR MANUAL EMAIL CHECK block gives the UCD email, Application No, Pre-Application No, company name, BRNs and the approval timestamp used below.
 1. In Mailtrap, search for chain CH4's UCD email.
 2. Open the guideline email; check To/CC, subject and body against TS01–TS03 and TS05.</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="G25" s="2" t="inlineStr">
         <is>
           <t>Ensure:
 • Combined Email Template 1 received with CH4's values; To = UCD email, CC = apply@eauto.my, Appointment Letter attached.</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr">
+      <c r="H25" s="2" t="inlineStr">
         <is>
           <t>LLP, 4 partners → the same combined guideline email
 Business-type coverage for 'the same email is sent to every UCD' (SRD §2.2.2).</t>
         </is>
       </c>
-      <c r="I24" s="2" t="inlineStr">
+      <c r="I25" s="2" t="inlineStr">
         <is>
           <t>12341_CH4</t>
-        </is>
-      </c>
-      <c r="J24" s="2" t="inlineStr">
-        <is>
-          <t>REQ-005</t>
-        </is>
-      </c>
-      <c r="K24" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="L24" s="2" t="inlineStr">
-        <is>
-          <t>Functional / Positive</t>
-        </is>
-      </c>
-      <c r="M24" s="2" t="inlineStr"/>
-      <c r="N24" s="2" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="O24" s="2" t="inlineStr"/>
-    </row>
-    <row r="25" ht="92" customHeight="1">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>12341_TS10</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Business Trading (Sabah) or (Sarawak)</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>2 directors (typed)</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>All Malaysian</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>Email Template 1 (combined)</t>
-        </is>
-      </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>Precondition: chain 12341_CH5 has been executed by the automation up to Application Approved (see the 'Test Data &amp; Chains' sheet). The run log's READY FOR MANUAL EMAIL CHECK block gives the UCD email, Application No, Pre-Application No, company name, BRNs and the approval timestamp used below.
-1. In Mailtrap, search for chain CH5's UCD email.
-2. Open the guideline email; check To/CC, subject and body against TS01–TS03 and TS05.</t>
-        </is>
-      </c>
-      <c r="G25" s="2" t="inlineStr">
-        <is>
-          <t>Ensure:
-• Combined Email Template 1 received with CH5's values; To = UCD email, CC = apply@eauto.my, Appointment Letter attached.</t>
-        </is>
-      </c>
-      <c r="H25" s="2" t="inlineStr">
-        <is>
-          <t>Business Trading (non-SSM) → the same combined guideline email
-v1.1 had this case TBC (no SSM data for the determination). v1.3 removes the determination, and SRD §2.2.2 says the same email is sent to every UCD, so the expected result is now confirmed by the SRD.</t>
-        </is>
-      </c>
-      <c r="I25" s="2" t="inlineStr">
-        <is>
-          <t>12341_CH5</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
@@ -1506,40 +1506,114 @@
       </c>
       <c r="O25" s="2" t="inlineStr"/>
     </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
+    <row r="26" ht="92" customHeight="1">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>12341_TS10</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Per chain</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Per chain</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Per chain</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Email Template 1 (combined)</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Precondition: chains CH5 (Sabah) and CH7 (Sarawak) executed to Application Approved.
+For each of CH5 and CH7:
+1. In Mailtrap, search for the chain's UCD email.
+2. Open the guideline email; check To/CC, subject and body against TS01–TS03 and TS05.</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Ensure:
+• For both: combined Email Template 1 received with that chain's values; To = UCD email, CC = apply@eauto.my, Appointment Letter attached.</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Business Trading (Sabah) and Business Trading (Sarawak) (non-SSM) → the same combined guideline email
+v1.1 had this case TBC (no SSM data for the determination). v1.3 removes the determination, and SRD §2.2.2 says the same email is sent to every UCD, so the expected result is now confirmed by the SRD.</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>12341_CH5, CH7</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>REQ-005</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>Functional / Positive</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr"/>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
         <is>
           <t>C — Appointment Letter email to RHB Support (Email Template 3)</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="92" customHeight="1">
-      <c r="A27" s="5" t="inlineStr">
+    <row r="28" ht="92" customHeight="1">
+      <c r="A28" s="5" t="inlineStr">
         <is>
           <t>12341_TS11</t>
         </is>
       </c>
-      <c r="B27" s="2" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
         <is>
           <t>Sole Proprietorship / Partnership</t>
         </is>
       </c>
-      <c r="C27" s="2" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr">
         <is>
           <t>4 business owners</t>
         </is>
       </c>
-      <c r="D27" s="2" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>All Malaysian</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>Email Template 3</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>Precondition: chain 12341_CH1 has been executed by the automation up to Application Approved (see the 'Test Data &amp; Chains' sheet). The run log's READY FOR MANUAL EMAIL CHECK block gives the UCD email, Application No, Pre-Application No, company name, BRNs and the approval timestamp used below.
 1. In Mailtrap, search for the UCD email address from the run log (it is in CC of this email).
@@ -1547,7 +1621,7 @@
 3. Inspect To and CC.</t>
         </is>
       </c>
-      <c r="G27" s="2" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>Ensure:
 • To: BIS.Support@rhbgroup.com.
@@ -1555,141 +1629,141 @@
 • Received after the Application approval timestamp.</t>
         </is>
       </c>
-      <c r="H27" s="2" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr">
         <is>
           <t>Appointment Letter email: To = BIS.Support@rhbgroup.com, CC = UCD email + apply@eauto.my
 Staging mail must be captured by Mailtrap so nothing reaches RHB — confirm (Q-17). Do not assert From (Q-12).</t>
         </is>
       </c>
-      <c r="I27" s="2" t="inlineStr">
+      <c r="I28" s="2" t="inlineStr">
         <is>
           <t>12341_CH1</t>
         </is>
       </c>
-      <c r="J27" s="2" t="inlineStr">
+      <c r="J28" s="2" t="inlineStr">
         <is>
           <t>REQ-006</t>
         </is>
       </c>
-      <c r="K27" s="2" t="inlineStr">
+      <c r="K28" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="L27" s="2" t="inlineStr">
+      <c r="L28" s="2" t="inlineStr">
         <is>
           <t>Functional / Positive</t>
         </is>
       </c>
-      <c r="M27" s="2" t="inlineStr"/>
-      <c r="N27" s="2" t="inlineStr">
+      <c r="M28" s="2" t="inlineStr"/>
+      <c r="N28" s="2" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O27" s="2" t="inlineStr"/>
-    </row>
-    <row r="28" ht="92" customHeight="1">
-      <c r="A28" s="5" t="inlineStr">
+      <c r="O28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29" ht="92" customHeight="1">
+      <c r="A29" s="5" t="inlineStr">
         <is>
           <t>12341_TS12</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>Sole Proprietorship / Partnership</t>
         </is>
       </c>
-      <c r="C28" s="2" t="inlineStr">
+      <c r="C29" s="2" t="inlineStr">
         <is>
           <t>4 business owners</t>
         </is>
       </c>
-      <c r="D28" s="2" t="inlineStr">
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>All Malaysian</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>Email Template 3</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="F29" s="2" t="inlineStr">
         <is>
           <t>Precondition: chain 12341_CH1 has been executed by the automation up to Application Approved (see the 'Test Data &amp; Chains' sheet). The run log's READY FOR MANUAL EMAIL CHECK block gives the UCD email, Application No, Pre-Application No, company name, BRNs and the approval timestamp used below.
 1. Open the email from TS11.
 2. Read the subject line.</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="G29" s="2" t="inlineStr">
         <is>
           <t>Ensure:
 • Subject = 'Approved eAuto Registration - [Company Name] - [BRN Number]' with [Company Name] = company name in the Application and [BRN Number] = the BRN agreed in Q-05.
   e.g. 'Approved eAuto Registration - ABC Motors Sdn Bhd - 202401234567'.</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr">
+      <c r="H29" s="2" t="inlineStr">
         <is>
           <t>Appointment Letter email subject with real values
 The SRD example uses a 12-digit number (new BRN format) but the field is not defined — Q-05. Record which BRN is shown.</t>
         </is>
       </c>
-      <c r="I28" s="2" t="inlineStr">
+      <c r="I29" s="2" t="inlineStr">
         <is>
           <t>12341_CH1</t>
         </is>
       </c>
-      <c r="J28" s="2" t="inlineStr">
+      <c r="J29" s="2" t="inlineStr">
         <is>
           <t>REQ-009</t>
         </is>
       </c>
-      <c r="K28" s="2" t="inlineStr">
+      <c r="K29" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="L28" s="2" t="inlineStr">
+      <c r="L29" s="2" t="inlineStr">
         <is>
           <t>Functional / Content</t>
         </is>
       </c>
-      <c r="M28" s="2" t="inlineStr"/>
-      <c r="N28" s="2" t="inlineStr">
+      <c r="M29" s="2" t="inlineStr"/>
+      <c r="N29" s="2" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O28" s="2" t="inlineStr"/>
-    </row>
-    <row r="29" ht="92" customHeight="1">
-      <c r="A29" s="5" t="inlineStr">
+      <c r="O29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30" ht="92" customHeight="1">
+      <c r="A30" s="5" t="inlineStr">
         <is>
           <t>12341_TS13</t>
         </is>
       </c>
-      <c r="B29" s="2" t="inlineStr">
+      <c r="B30" s="2" t="inlineStr">
         <is>
           <t>Sole Proprietorship / Partnership</t>
         </is>
       </c>
-      <c r="C29" s="2" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t>4 business owners</t>
         </is>
       </c>
-      <c r="D29" s="2" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>All Malaysian</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>Email Template 3</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr">
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>Precondition: chain 12341_CH1 has been executed by the automation up to Application Approved (see the 'Test Data &amp; Chains' sheet). The run log's READY FOR MANUAL EMAIL CHECK block gives the UCD email, Application No, Pre-Application No, company name, BRNs and the approval timestamp used below.
 1. Open the email body.
@@ -1697,7 +1771,7 @@
 3. Compare each value line with the run log / Application.</t>
         </is>
       </c>
-      <c r="G29" s="2" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>Ensure:
 • Every paragraph is present, in order, with the same wording, including the one (1) working day request, the Reply All instruction and the signature block.
@@ -1705,221 +1779,221 @@
 • The withdrawn sentence 'The above company is not eligible for RHB's online account-opening process and will complete the account opening at an RHB branch.' does NOT appear.</t>
         </is>
       </c>
-      <c r="H29" s="2" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr">
         <is>
           <t>Appointment Letter email body matches Email Template 3 word for word, with correct values
 SRD v1.3 §2.2.5.1. The chain uses different name / mobile / email for the Admin In Charge and the Director in Charge so the email shows which source the system used (Q-04).</t>
         </is>
       </c>
-      <c r="I29" s="2" t="inlineStr">
+      <c r="I30" s="2" t="inlineStr">
         <is>
           <t>12341_CH1</t>
         </is>
       </c>
-      <c r="J29" s="2" t="inlineStr">
+      <c r="J30" s="2" t="inlineStr">
         <is>
           <t>REQ-009</t>
         </is>
       </c>
-      <c r="K29" s="2" t="inlineStr">
+      <c r="K30" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="L29" s="2" t="inlineStr">
+      <c r="L30" s="2" t="inlineStr">
         <is>
           <t>Functional / Content</t>
         </is>
       </c>
-      <c r="M29" s="2" t="inlineStr"/>
-      <c r="N29" s="2" t="inlineStr">
+      <c r="M30" s="2" t="inlineStr"/>
+      <c r="N30" s="2" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O29" s="2" t="inlineStr"/>
-    </row>
-    <row r="30" ht="92" customHeight="1">
-      <c r="A30" s="5" t="inlineStr">
+      <c r="O30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31" ht="92" customHeight="1">
+      <c r="A31" s="5" t="inlineStr">
         <is>
           <t>12341_TS14</t>
         </is>
       </c>
-      <c r="B30" s="2" t="inlineStr">
+      <c r="B31" s="2" t="inlineStr">
         <is>
           <t>Sole Proprietorship / Partnership</t>
         </is>
       </c>
-      <c r="C30" s="2" t="inlineStr">
+      <c r="C31" s="2" t="inlineStr">
         <is>
           <t>4 business owners</t>
         </is>
       </c>
-      <c r="D30" s="2" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>All Malaysian</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="E31" s="2" t="inlineStr">
         <is>
           <t>Email Template 3</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="F31" s="2" t="inlineStr">
         <is>
           <t>Precondition: chain 12341_CH1 has been executed by the automation up to Application Approved (see the 'Test Data &amp; Chains' sheet). The run log's READY FOR MANUAL EMAIL CHECK block gives the UCD email, Application No, Pre-Application No, company name, BRNs and the approval timestamp used below.
 1. In the email from TS11, open Attachments.
 2. Download and open the attachment.</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="G31" s="2" t="inlineStr">
         <is>
           <t>Ensure:
 • Exactly one Appointment Letter attachment, opens without error, for THIS Application.</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr">
+      <c r="H31" s="2" t="inlineStr">
         <is>
           <t>Appointment Letter is attached to the RHB Support email</t>
         </is>
       </c>
-      <c r="I30" s="2" t="inlineStr">
+      <c r="I31" s="2" t="inlineStr">
         <is>
           <t>12341_CH1</t>
         </is>
       </c>
-      <c r="J30" s="2" t="inlineStr">
+      <c r="J31" s="2" t="inlineStr">
         <is>
           <t>REQ-008</t>
         </is>
       </c>
-      <c r="K30" s="2" t="inlineStr">
+      <c r="K31" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="L30" s="2" t="inlineStr">
+      <c r="L31" s="2" t="inlineStr">
         <is>
           <t>Functional / Positive</t>
         </is>
       </c>
-      <c r="M30" s="2" t="inlineStr"/>
-      <c r="N30" s="2" t="inlineStr">
+      <c r="M31" s="2" t="inlineStr"/>
+      <c r="N31" s="2" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O30" s="2" t="inlineStr"/>
-    </row>
-    <row r="31" ht="105" customHeight="1">
-      <c r="A31" s="5" t="inlineStr">
+      <c r="O31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32" ht="105" customHeight="1">
+      <c r="A32" s="5" t="inlineStr">
         <is>
           <t>12341_TS15</t>
         </is>
       </c>
-      <c r="B31" s="2" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>Per chain</t>
         </is>
       </c>
-      <c r="C31" s="2" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
         <is>
           <t>Per chain</t>
         </is>
       </c>
-      <c r="D31" s="2" t="inlineStr">
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>Per chain</t>
         </is>
       </c>
-      <c r="E31" s="2" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr">
         <is>
           <t>Email Template 3</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>Precondition: chains CH2, CH3, CH4 and CH5 executed to Application Approved.
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Precondition: chains CH2, CH3, CH4, CH5, CH7 and CH8 executed to Application Approved.
 For each chain:
 1. In Mailtrap, search for the chain's UCD email.
 2. Open the 'Approved eAuto Registration' email.
 3. Check To/CC, subject, body values and the attachment as in TS11–TS14.</t>
         </is>
       </c>
-      <c r="G31" s="2" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>Ensure:
 • For every chain: one Appointment Letter email, To = BIS.Support@rhbgroup.com, CC = UCD email + apply@eauto.my, subject/body per Email Template 3 with that chain's values, Appointment Letter attached.</t>
         </is>
       </c>
-      <c r="H31" s="2" t="inlineStr">
+      <c r="H32" s="2" t="inlineStr">
         <is>
           <t>Appointment Letter email is sent for every approved Application, whatever the company structure
-Business Trading (CH5): what [BRN Number] shows is Q-05 / Q-09 — record it.</t>
-        </is>
-      </c>
-      <c r="I31" s="2" t="inlineStr">
-        <is>
-          <t>12341_CH2, CH3, CH4, CH5</t>
-        </is>
-      </c>
-      <c r="J31" s="2" t="inlineStr">
+Business Trading (CH5, CH7): what [BRN Number] shows is Q-05 / Q-09 — record it.</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>12341_CH2, CH3, CH4, CH5, CH7, CH8</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
         <is>
           <t>REQ-006, REQ-009</t>
         </is>
       </c>
-      <c r="K31" s="2" t="inlineStr">
+      <c r="K32" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="L31" s="2" t="inlineStr">
+      <c r="L32" s="2" t="inlineStr">
         <is>
           <t>Functional / Positive</t>
         </is>
       </c>
-      <c r="M31" s="2" t="inlineStr"/>
-      <c r="N31" s="2" t="inlineStr">
+      <c r="M32" s="2" t="inlineStr"/>
+      <c r="N32" s="2" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O31" s="2" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="4" t="inlineStr">
+      <c r="O32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
         <is>
           <t>D — Appointment Letter document</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="131" customHeight="1">
-      <c r="A33" s="5" t="inlineStr">
+    <row r="34" ht="131" customHeight="1">
+      <c r="A34" s="5" t="inlineStr">
         <is>
           <t>12341_TS16</t>
         </is>
       </c>
-      <c r="B33" s="2" t="inlineStr">
+      <c r="B34" s="2" t="inlineStr">
         <is>
           <t>Sole Proprietorship / Partnership</t>
         </is>
       </c>
-      <c r="C33" s="2" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>4 business owners</t>
         </is>
       </c>
-      <c r="D33" s="2" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>All Malaysian</t>
         </is>
       </c>
-      <c r="E33" s="2" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>Appointment Letter</t>
         </is>
       </c>
-      <c r="F33" s="2" t="inlineStr">
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>Precondition: chain 12341_CH1 has been executed by the automation up to Application Approved (see the 'Test Data &amp; Chains' sheet). The run log's READY FOR MANUAL EMAIL CHECK block gives the UCD email, Application No, Pre-Application No, company name, BRNs and the approval timestamp used below.
 1. Open the Appointment Letter attached to the UCD email (TS05).
@@ -1927,7 +2001,7 @@
 3. Check page header, body, signatory and footer on every page.</t>
         </is>
       </c>
-      <c r="G33" s="2" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>Ensure:
 • Title: 'LETTER OF CONFIRMATION OF REGISTRATION AS A USED CAR DEALER (UCD) UNDER eAUTO SDN. BHD. PLATFORM'.
@@ -1939,67 +2013,67 @@
 • No layout break (text cut off, overlapping, blank page).</t>
         </is>
       </c>
-      <c r="H33" s="2" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr">
         <is>
           <t>Appointment Letter layout and fixed text match the SRD template
 SRD v1.3 §2.2.5.2 items 1–8. Title spacing differs between the SRD ('SDN. BHD. PLATFORM') and the template .docx ('SDN. BHD.PLATFORM') — Q-10.</t>
         </is>
       </c>
-      <c r="I33" s="2" t="inlineStr">
+      <c r="I34" s="2" t="inlineStr">
         <is>
           <t>12341_CH1</t>
         </is>
       </c>
-      <c r="J33" s="2" t="inlineStr">
+      <c r="J34" s="2" t="inlineStr">
         <is>
           <t>REQ-007</t>
         </is>
       </c>
-      <c r="K33" s="2" t="inlineStr">
+      <c r="K34" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="L33" s="2" t="inlineStr">
+      <c r="L34" s="2" t="inlineStr">
         <is>
           <t>Functional / Content</t>
         </is>
       </c>
-      <c r="M33" s="2" t="inlineStr"/>
-      <c r="N33" s="2" t="inlineStr">
+      <c r="M34" s="2" t="inlineStr"/>
+      <c r="N34" s="2" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O33" s="2" t="inlineStr"/>
-    </row>
-    <row r="34" ht="170" customHeight="1">
-      <c r="A34" s="5" t="inlineStr">
+      <c r="O34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35" ht="170" customHeight="1">
+      <c r="A35" s="5" t="inlineStr">
         <is>
           <t>12341_TS17</t>
         </is>
       </c>
-      <c r="B34" s="2" t="inlineStr">
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>Sole Proprietorship / Partnership</t>
         </is>
       </c>
-      <c r="C34" s="2" t="inlineStr">
+      <c r="C35" s="2" t="inlineStr">
         <is>
           <t>4 business owners</t>
         </is>
       </c>
-      <c r="D34" s="2" t="inlineStr">
+      <c r="D35" s="2" t="inlineStr">
         <is>
           <t>All Malaysian</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="E35" s="2" t="inlineStr">
         <is>
           <t>Appointment Letter</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="F35" s="2" t="inlineStr">
         <is>
           <t>Precondition: chain 12341_CH1 has been executed by the automation up to Application Approved (see the 'Test Data &amp; Chains' sheet). The run log's READY FOR MANUAL EMAIL CHECK block gives the UCD email, Application No, Pre-Application No, company name, BRNs and the approval timestamp used below.
 1. Open the Appointment Letter.
@@ -2013,7 +2087,7 @@
    g. Clause 4 table: UCD Name, Company Registration No., UCD / Dealer Reference No.</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="G35" s="2" t="inlineStr">
         <is>
           <t>Ensure:
 • Date = approval date in DD/MM/YYYY.
@@ -2025,146 +2099,146 @@
 • No placeholder (text in [ ]) remains unresolved.</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr">
+      <c r="H35" s="2" t="inlineStr">
         <is>
           <t>Appointment Letter pre-populated fields carry the approved Application's data without manual input
 SRD v1.3 §2.2.5.2 item 9. The sample letter keeps square brackets around Our Ref and around the registration no. in the recipient block and Clause 1 but not in the table — Q-07.</t>
         </is>
       </c>
-      <c r="I34" s="2" t="inlineStr">
+      <c r="I35" s="2" t="inlineStr">
         <is>
           <t>12341_CH1</t>
         </is>
       </c>
-      <c r="J34" s="2" t="inlineStr">
+      <c r="J35" s="2" t="inlineStr">
         <is>
           <t>REQ-007</t>
         </is>
       </c>
-      <c r="K34" s="2" t="inlineStr">
+      <c r="K35" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="L34" s="2" t="inlineStr">
+      <c r="L35" s="2" t="inlineStr">
         <is>
           <t>Functional / Data</t>
         </is>
       </c>
-      <c r="M34" s="2" t="inlineStr"/>
-      <c r="N34" s="2" t="inlineStr">
+      <c r="M35" s="2" t="inlineStr"/>
+      <c r="N35" s="2" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O34" s="2" t="inlineStr"/>
-    </row>
-    <row r="35" ht="92" customHeight="1">
-      <c r="A35" s="5" t="inlineStr">
+      <c r="O35" s="2" t="inlineStr"/>
+    </row>
+    <row r="36" ht="92" customHeight="1">
+      <c r="A36" s="5" t="inlineStr">
         <is>
           <t>12341_TS18</t>
         </is>
       </c>
-      <c r="B35" s="2" t="inlineStr">
+      <c r="B36" s="2" t="inlineStr">
         <is>
           <t>Sole Proprietorship / Partnership</t>
         </is>
       </c>
-      <c r="C35" s="2" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
         <is>
           <t>4 business owners</t>
         </is>
       </c>
-      <c r="D35" s="2" t="inlineStr">
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>All Malaysian</t>
         </is>
       </c>
-      <c r="E35" s="2" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>Appointment Letter</t>
         </is>
       </c>
-      <c r="F35" s="2" t="inlineStr">
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>Precondition: chain 12341_CH1 has been executed by the automation up to Application Approved (see the 'Test Data &amp; Chains' sheet). The run log's READY FOR MANUAL EMAIL CHECK block gives the UCD email, Application No, Pre-Application No, company name, BRNs and the approval timestamp used below.
 1. Download the attachment from the UCD guideline email (TS05) and from the RHB Support email (TS14).
 2. Compare file name, size and content.</t>
         </is>
       </c>
-      <c r="G35" s="2" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>Ensure:
 • Both attachments are the same letter (same Our Ref, date, company, BRNs, reference numbers).</t>
         </is>
       </c>
-      <c r="H35" s="2" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr">
         <is>
           <t>The same Appointment Letter is attached to both emails</t>
         </is>
       </c>
-      <c r="I35" s="2" t="inlineStr">
+      <c r="I36" s="2" t="inlineStr">
         <is>
           <t>12341_CH1</t>
         </is>
       </c>
-      <c r="J35" s="2" t="inlineStr">
+      <c r="J36" s="2" t="inlineStr">
         <is>
           <t>REQ-008</t>
         </is>
       </c>
-      <c r="K35" s="2" t="inlineStr">
+      <c r="K36" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="L35" s="2" t="inlineStr">
+      <c r="L36" s="2" t="inlineStr">
         <is>
           <t>Functional / Data</t>
         </is>
       </c>
-      <c r="M35" s="2" t="inlineStr"/>
-      <c r="N35" s="2" t="inlineStr">
+      <c r="M36" s="2" t="inlineStr"/>
+      <c r="N36" s="2" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O35" s="2" t="inlineStr"/>
-    </row>
-    <row r="36" ht="92" customHeight="1">
-      <c r="A36" s="5" t="inlineStr">
+      <c r="O36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37" ht="92" customHeight="1">
+      <c r="A37" s="5" t="inlineStr">
         <is>
           <t>12341_TS19</t>
         </is>
       </c>
-      <c r="B36" s="2" t="inlineStr">
+      <c r="B37" s="2" t="inlineStr">
         <is>
           <t>Per chain</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr">
+      <c r="C37" s="2" t="inlineStr">
         <is>
           <t>Per chain</t>
         </is>
       </c>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="D37" s="2" t="inlineStr">
         <is>
           <t>Per chain</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="E37" s="2" t="inlineStr">
         <is>
           <t>Appointment Letter</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr">
-        <is>
-          <t>Precondition: chains CH3 and CH4 executed to Application Approved.
-1. Open the Appointment Letter of CH3 (Sdn Bhd) and of CH4 (LLP).
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Precondition: chains CH3, CH8 and CH4 executed to Application Approved.
+1. Open the Appointment Letter of CH3 and CH8 (Sdn Bhd) and of CH4 (LLP).
 2. Check the registration number in the recipient block, Clause 1 and Clause 4 against the SSM details of each Pre-Application.</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="G37" s="2" t="inlineStr">
         <is>
           <t>Ensure:
 • Sdn Bhd: '&lt;old ROC with check letter&gt; (&lt;12-digit new ROC&gt;)', e.g. '639691-H (200401001188)'.
@@ -2172,141 +2246,141 @@
 • Values identical to the Pre-Application summary SSM details; nothing truncated or doubled (e.g. no '-H-A').</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr">
+      <c r="H37" s="2" t="inlineStr">
         <is>
           <t>Appointment Letter registration number for Sdn Bhd and LLP formats
 The 24.09 run showed eAuto can render a doubled check letter ('IP0581553-U-A') when eSim is seeded whole — the chain now seeds split; this check catches a regression of that in the letter.</t>
         </is>
       </c>
-      <c r="I36" s="2" t="inlineStr">
-        <is>
-          <t>12341_CH3, CH4</t>
-        </is>
-      </c>
-      <c r="J36" s="2" t="inlineStr">
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>12341_CH3, CH4, CH8</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
         <is>
           <t>REQ-007</t>
         </is>
       </c>
-      <c r="K36" s="2" t="inlineStr">
+      <c r="K37" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="L36" s="2" t="inlineStr">
+      <c r="L37" s="2" t="inlineStr">
         <is>
           <t>Functional / Data</t>
         </is>
       </c>
-      <c r="M36" s="2" t="inlineStr"/>
-      <c r="N36" s="2" t="inlineStr">
+      <c r="M37" s="2" t="inlineStr"/>
+      <c r="N37" s="2" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O36" s="2" t="inlineStr"/>
-    </row>
-    <row r="37" ht="92" customHeight="1">
-      <c r="A37" s="6" t="inlineStr">
+      <c r="O37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38" ht="92" customHeight="1">
+      <c r="A38" s="6" t="inlineStr">
         <is>
           <t>12341_TS20</t>
         </is>
       </c>
-      <c r="B37" s="2" t="inlineStr">
-        <is>
-          <t>Business Trading (Sabah) or (Sarawak)</t>
-        </is>
-      </c>
-      <c r="C37" s="2" t="inlineStr">
-        <is>
-          <t>2 directors (typed)</t>
-        </is>
-      </c>
-      <c r="D37" s="2" t="inlineStr">
-        <is>
-          <t>All Malaysian</t>
-        </is>
-      </c>
-      <c r="E37" s="2" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Per chain</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>Per chain</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Per chain</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
         <is>
           <t>Appointment Letter</t>
         </is>
       </c>
-      <c r="F37" s="2" t="inlineStr">
-        <is>
-          <t>Precondition: chain 12341_CH5 has been executed by the automation up to Application Approved (see the 'Test Data &amp; Chains' sheet). The run log's READY FOR MANUAL EMAIL CHECK block gives the UCD email, Application No, Pre-Application No, company name, BRNs and the approval timestamp used below.
-1. Open the Appointment Letter of CH5.
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Precondition: chains CH5 and CH7 executed to Application Approved.
+1. Open the Appointment Letter of CH5 and of CH7.
 2. Check the recipient block, Clause 1 and Clause 4 'Company Registration No.'.</t>
         </is>
       </c>
-      <c r="G37" s="2" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>Ensure:
 • TBC — the SRD sources [Old BRN] / [New BRN] from the SSM details, which a Business Trading company does not have (Q-09).
 • In any case: the letter is generated and attached, and contains no unresolved placeholder or empty brackets such as '()'.</t>
         </is>
       </c>
-      <c r="H37" s="2" t="inlineStr">
-        <is>
-          <t>Appointment Letter for a Business Trading (non-SSM) company
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Appointment Letter for a Business Trading (non-SSM) company — Sabah and Sarawak
 RED — expected result pending Q-09.</t>
         </is>
       </c>
-      <c r="I37" s="2" t="inlineStr">
-        <is>
-          <t>12341_CH5</t>
-        </is>
-      </c>
-      <c r="J37" s="2" t="inlineStr">
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>12341_CH5, CH7</t>
+        </is>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
         <is>
           <t>REQ-007</t>
         </is>
       </c>
-      <c r="K37" s="2" t="inlineStr">
+      <c r="K38" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="L37" s="2" t="inlineStr">
+      <c r="L38" s="2" t="inlineStr">
         <is>
           <t>Functional / Data</t>
         </is>
       </c>
-      <c r="M37" s="2" t="inlineStr"/>
-      <c r="N37" s="2" t="inlineStr">
+      <c r="M38" s="2" t="inlineStr"/>
+      <c r="N38" s="2" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O37" s="2" t="inlineStr"/>
-    </row>
-    <row r="38" ht="92" customHeight="1">
-      <c r="A38" s="5" t="inlineStr">
+      <c r="O38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39" ht="92" customHeight="1">
+      <c r="A39" s="5" t="inlineStr">
         <is>
           <t>12341_TS21</t>
         </is>
       </c>
-      <c r="B38" s="2" t="inlineStr">
+      <c r="B39" s="2" t="inlineStr">
         <is>
           <t>Per chain</t>
         </is>
       </c>
-      <c r="C38" s="2" t="inlineStr">
+      <c r="C39" s="2" t="inlineStr">
         <is>
           <t>Per chain</t>
         </is>
       </c>
-      <c r="D38" s="2" t="inlineStr">
+      <c r="D39" s="2" t="inlineStr">
         <is>
           <t>Per chain</t>
         </is>
       </c>
-      <c r="E38" s="2" t="inlineStr">
+      <c r="E39" s="2" t="inlineStr">
         <is>
           <t>Appointment Letter</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="F39" s="2" t="inlineStr">
         <is>
           <t>Precondition: chain 12341_CH1 has been executed by the automation up to Application Approved (see the 'Test Data &amp; Chains' sheet). The run log's READY FOR MANUAL EMAIL CHECK block gives the UCD email, Application No, Pre-Application No, company name, BRNs and the approval timestamp used below.
 1. In each email (guideline + RHB Support) search the subject and body for '[' and ']'.
@@ -2314,302 +2388,302 @@
 3. Repeat for every chain executed.</t>
         </is>
       </c>
-      <c r="G38" s="2" t="inlineStr">
+      <c r="G39" s="2" t="inlineStr">
         <is>
           <t>Ensure:
 • None of these appear literally: [Application No], [Company Name], [BRN Number], [Name], [Contact Number], [UCD Email Address], [RHB Online Registration Link], [Application Link], [DD/MM/YYYY], [YYYY], [UCD Company Name], [Old BRN], [New BRN], [Company Address], [Pre-Application No].
 • No empty value (e.g. 'Company Name: ' with nothing after it).</t>
         </is>
       </c>
-      <c r="H38" s="2" t="inlineStr">
+      <c r="H39" s="2" t="inlineStr">
         <is>
           <t>No unresolved placeholders in any subject, body or letter
 Brackets kept around a resolved value in the letter (Our Ref, registration no.) are Q-07, not a placeholder failure.</t>
         </is>
       </c>
-      <c r="I38" s="2" t="inlineStr">
+      <c r="I39" s="2" t="inlineStr">
         <is>
           <t>12341_CH1 (and every chain)</t>
         </is>
       </c>
-      <c r="J38" s="2" t="inlineStr">
+      <c r="J39" s="2" t="inlineStr">
         <is>
           <t>REQ-005, REQ-007, REQ-009</t>
         </is>
       </c>
-      <c r="K38" s="2" t="inlineStr">
+      <c r="K39" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="L38" s="2" t="inlineStr">
+      <c r="L39" s="2" t="inlineStr">
         <is>
           <t>Functional / Content</t>
         </is>
       </c>
-      <c r="M38" s="2" t="inlineStr"/>
-      <c r="N38" s="2" t="inlineStr">
+      <c r="M39" s="2" t="inlineStr"/>
+      <c r="N39" s="2" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O38" s="2" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="4" t="inlineStr">
+      <c r="O39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
         <is>
           <t>E — Trigger, suppression and regression</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="92" customHeight="1">
-      <c r="A40" s="5" t="inlineStr">
+    <row r="41" ht="92" customHeight="1">
+      <c r="A41" s="5" t="inlineStr">
         <is>
           <t>12341_TS22</t>
         </is>
       </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="B41" s="2" t="inlineStr">
         <is>
           <t>Sole Proprietorship / Partnership</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr">
+      <c r="C41" s="2" t="inlineStr">
         <is>
           <t>4 business owners</t>
         </is>
       </c>
-      <c r="D40" s="2" t="inlineStr">
+      <c r="D41" s="2" t="inlineStr">
         <is>
           <t>All Malaysian</t>
         </is>
       </c>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="E41" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="F41" s="2" t="inlineStr">
         <is>
           <t>Precondition: chain 12341_CH1 has been executed by the automation up to Application Approved (see the 'Test Data &amp; Chains' sheet). The run log's READY FOR MANUAL EMAIL CHECK block gives the UCD email, Application No, Pre-Application No, company name, BRNs and the approval timestamp used below.
 1. In Mailtrap, list every email to the UCD email address of CH1.
 2. Look for the existing approved-application email (the one that carried the Offer Letter, Direct Debit Application form and Board of Resolution) — use the production subject from a pre-CR approval as reference (Q-23).</t>
         </is>
       </c>
-      <c r="G40" s="2" t="inlineStr">
+      <c r="G41" s="2" t="inlineStr">
         <is>
           <t>Ensure:
 • The old approved-application email is not received.
 • No email from eAuto on this approval carries the Offer Letter, Direct Debit Application form or Board of Resolution.</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr">
+      <c r="H41" s="2" t="inlineStr">
         <is>
           <t>Old approved-application email (3 RHB documents) is no longer sent
 Negative assertion — passes silently if only the arriving emails are looked at. Needs the old email's subject (Q-23).</t>
         </is>
       </c>
-      <c r="I40" s="2" t="inlineStr">
+      <c r="I41" s="2" t="inlineStr">
         <is>
           <t>12341_CH1</t>
         </is>
       </c>
-      <c r="J40" s="2" t="inlineStr">
+      <c r="J41" s="2" t="inlineStr">
         <is>
           <t>REQ-001</t>
         </is>
       </c>
-      <c r="K40" s="2" t="inlineStr">
+      <c r="K41" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="L40" s="2" t="inlineStr">
+      <c r="L41" s="2" t="inlineStr">
         <is>
           <t>Regression / Negative</t>
         </is>
       </c>
-      <c r="M40" s="2" t="inlineStr"/>
-      <c r="N40" s="2" t="inlineStr">
+      <c r="M41" s="2" t="inlineStr"/>
+      <c r="N41" s="2" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O40" s="2" t="inlineStr"/>
-    </row>
-    <row r="41" ht="92" customHeight="1">
-      <c r="A41" s="5" t="inlineStr">
+      <c r="O41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42" ht="92" customHeight="1">
+      <c r="A42" s="5" t="inlineStr">
         <is>
           <t>12341_TS23</t>
         </is>
       </c>
-      <c r="B41" s="2" t="inlineStr">
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>Sole Proprietorship / Partnership</t>
         </is>
       </c>
-      <c r="C41" s="2" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr">
         <is>
           <t>4 business owners</t>
         </is>
       </c>
-      <c r="D41" s="2" t="inlineStr">
+      <c r="D42" s="2" t="inlineStr">
         <is>
           <t>All Malaysian</t>
         </is>
       </c>
-      <c r="E41" s="2" t="inlineStr">
+      <c r="E42" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F41" s="2" t="inlineStr">
+      <c r="F42" s="2" t="inlineStr">
         <is>
           <t>Precondition: chain 12341_CH1 has been executed by the automation up to Application Approved (see the 'Test Data &amp; Chains' sheet). The run log's READY FOR MANUAL EMAIL CHECK block gives the UCD email, Application No, Pre-Application No, company name, BRNs and the approval timestamp used below.
 1. In Mailtrap, list every email for CH1's UCD email address received from the Application approval time until the quiet window has passed (Q-16).
 2. Count emails by subject.</t>
         </is>
       </c>
-      <c r="G41" s="2" t="inlineStr">
+      <c r="G42" s="2" t="inlineStr">
         <is>
           <t>Ensure:
 • Exactly 1 × 'RHB Online / Branch Account Opening - …' and exactly 1 × 'Approved eAuto Registration - …'.
 • No other new email triggered by the approval (apart from any existing, unchanged notification — list it if one appears).</t>
         </is>
       </c>
-      <c r="H41" s="2" t="inlineStr">
+      <c r="H42" s="2" t="inlineStr">
         <is>
           <t>One approval sends exactly one guideline email and one Appointment Letter email (no duplicates)</t>
         </is>
       </c>
-      <c r="I41" s="2" t="inlineStr">
+      <c r="I42" s="2" t="inlineStr">
         <is>
           <t>12341_CH1</t>
         </is>
       </c>
-      <c r="J41" s="2" t="inlineStr">
+      <c r="J42" s="2" t="inlineStr">
         <is>
           <t>REQ-001</t>
         </is>
       </c>
-      <c r="K41" s="2" t="inlineStr">
+      <c r="K42" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="L41" s="2" t="inlineStr">
+      <c r="L42" s="2" t="inlineStr">
         <is>
           <t>Functional / Negative</t>
         </is>
       </c>
-      <c r="M41" s="2" t="inlineStr"/>
-      <c r="N41" s="2" t="inlineStr">
+      <c r="M42" s="2" t="inlineStr"/>
+      <c r="N42" s="2" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O41" s="2" t="inlineStr"/>
-    </row>
-    <row r="42" ht="92" customHeight="1">
-      <c r="A42" s="5" t="inlineStr">
+      <c r="O42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43" ht="92" customHeight="1">
+      <c r="A43" s="5" t="inlineStr">
         <is>
           <t>12341_TS24</t>
         </is>
       </c>
-      <c r="B42" s="2" t="inlineStr">
+      <c r="B43" s="2" t="inlineStr">
         <is>
           <t>Sole Proprietorship / Partnership</t>
         </is>
       </c>
-      <c r="C42" s="2" t="inlineStr">
+      <c r="C43" s="2" t="inlineStr">
         <is>
           <t>4 business owners</t>
         </is>
       </c>
-      <c r="D42" s="2" t="inlineStr">
+      <c r="D43" s="2" t="inlineStr">
         <is>
           <t>All Malaysian</t>
         </is>
       </c>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="E43" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F42" s="2" t="inlineStr">
+      <c r="F43" s="2" t="inlineStr">
         <is>
           <t>Precondition: chain 12341_CH1 has been executed by the automation up to Application Approved (see the 'Test Data &amp; Chains' sheet). The run log's READY FOR MANUAL EMAIL CHECK block gives the UCD email, Application No, Pre-Application No, company name, BRNs and the approval timestamp used below.
 1. From the run log, take the 'pre-application approved' timestamp and the 'application approved' timestamp.
 2. In Mailtrap, list emails for CH1's UCD email received between those two times.</t>
         </is>
       </c>
-      <c r="G42" s="2" t="inlineStr">
+      <c r="G43" s="2" t="inlineStr">
         <is>
           <t>Ensure:
 • No 'RHB Online / Branch Account Opening' or 'Approved eAuto Registration' email is received before the Application approval.
 • The existing Pre-Application approval email (Application Link) is still received as before.</t>
         </is>
       </c>
-      <c r="H42" s="2" t="inlineStr">
+      <c r="H43" s="2" t="inlineStr">
         <is>
           <t>Pre-Application approval does not send the new emails
 Gap noted by the previous QA (not in the v1.1 sheet). No extra test data: uses CH1's timestamps.</t>
         </is>
       </c>
-      <c r="I42" s="2" t="inlineStr">
+      <c r="I43" s="2" t="inlineStr">
         <is>
           <t>12341_CH1</t>
         </is>
       </c>
-      <c r="J42" s="2" t="inlineStr">
+      <c r="J43" s="2" t="inlineStr">
         <is>
           <t>REQ-001</t>
         </is>
       </c>
-      <c r="K42" s="2" t="inlineStr">
+      <c r="K43" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="L42" s="2" t="inlineStr">
+      <c r="L43" s="2" t="inlineStr">
         <is>
           <t>Functional / Negative</t>
         </is>
       </c>
-      <c r="M42" s="2" t="inlineStr"/>
-      <c r="N42" s="2" t="inlineStr">
+      <c r="M43" s="2" t="inlineStr"/>
+      <c r="N43" s="2" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O42" s="2" t="inlineStr"/>
-    </row>
-    <row r="43" ht="92" customHeight="1">
-      <c r="A43" s="5" t="inlineStr">
+      <c r="O43" s="2" t="inlineStr"/>
+    </row>
+    <row r="44" ht="92" customHeight="1">
+      <c r="A44" s="5" t="inlineStr">
         <is>
           <t>12341_TS25</t>
         </is>
       </c>
-      <c r="B43" s="2" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>Sole Proprietorship / Partnership</t>
         </is>
       </c>
-      <c r="C43" s="2" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr">
         <is>
           <t>4 business owners</t>
         </is>
       </c>
-      <c r="D43" s="2" t="inlineStr">
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>All Malaysian</t>
         </is>
       </c>
-      <c r="E43" s="2" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F43" s="2" t="inlineStr">
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>Precondition: chain 12341_CH6 has been executed by the automation up to Application Submitted (see the 'Test Data &amp; Chains' sheet). The run log's READY FOR MANUAL EMAIL CHECK block gives the UCD email, Application No, Pre-Application No, company name, BRNs and the approval timestamp used below.
 1. In Mailtrap, list emails for CH6's UCD email after the 'application submitted' timestamp; wait the quiet window (Q-16).
@@ -2617,7 +2691,7 @@
 3. In Mailtrap, list emails again after the revert; wait the quiet window.</t>
         </is>
       </c>
-      <c r="G43" s="2" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr">
         <is>
           <t>Ensure:
 • No guideline email and no Appointment Letter email after submission.
@@ -2625,67 +2699,67 @@
 • Existing revert notification (if any) unchanged.</t>
         </is>
       </c>
-      <c r="H43" s="2" t="inlineStr">
+      <c r="H44" s="2" t="inlineStr">
         <is>
           <t>No new email at Application Submitted, nor on Revert to UCD
 The trigger is Application approval only (REQ-001).</t>
         </is>
       </c>
-      <c r="I43" s="2" t="inlineStr">
+      <c r="I44" s="2" t="inlineStr">
         <is>
           <t>12341_CH6</t>
         </is>
       </c>
-      <c r="J43" s="2" t="inlineStr">
+      <c r="J44" s="2" t="inlineStr">
         <is>
           <t>REQ-001</t>
         </is>
       </c>
-      <c r="K43" s="2" t="inlineStr">
+      <c r="K44" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="L43" s="2" t="inlineStr">
+      <c r="L44" s="2" t="inlineStr">
         <is>
           <t>Functional / Negative</t>
         </is>
       </c>
-      <c r="M43" s="2" t="inlineStr"/>
-      <c r="N43" s="2" t="inlineStr">
+      <c r="M44" s="2" t="inlineStr"/>
+      <c r="N44" s="2" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O43" s="2" t="inlineStr"/>
-    </row>
-    <row r="44" ht="118" customHeight="1">
-      <c r="A44" s="5" t="inlineStr">
+      <c r="O44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45" ht="118" customHeight="1">
+      <c r="A45" s="5" t="inlineStr">
         <is>
           <t>12341_TS26</t>
         </is>
       </c>
-      <c r="B44" s="2" t="inlineStr">
+      <c r="B45" s="2" t="inlineStr">
         <is>
           <t>Sole Proprietorship / Partnership</t>
         </is>
       </c>
-      <c r="C44" s="2" t="inlineStr">
+      <c r="C45" s="2" t="inlineStr">
         <is>
           <t>4 business owners</t>
         </is>
       </c>
-      <c r="D44" s="2" t="inlineStr">
+      <c r="D45" s="2" t="inlineStr">
         <is>
           <t>All Malaysian</t>
         </is>
       </c>
-      <c r="E44" s="2" t="inlineStr">
+      <c r="E45" s="2" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F44" s="2" t="inlineStr">
+      <c r="F45" s="2" t="inlineStr">
         <is>
           <t>Precondition: chain 12341_CH1 has been executed by the automation up to Application Approved (see the 'Test Data &amp; Chains' sheet). The run log's READY FOR MANUAL EMAIL CHECK block gives the UCD email, Application No, Pre-Application No, company name, BRNs and the approval timestamp used below. Run AFTER TS01–TS24 so their mailbox counts are not disturbed.
 1. In BackOffice &gt; Application listing, search CH1's Application No and check its status.
@@ -2695,7 +2769,7 @@
 5. In Mailtrap, open the resubmission email.</t>
         </is>
       </c>
-      <c r="G44" s="2" t="inlineStr">
+      <c r="G45" s="2" t="inlineStr">
         <is>
           <t>Ensure:
 • Status shows Approved, as before the CR.
@@ -2704,39 +2778,39 @@
 • The Reverted Reason displays on the Registration Document page.</t>
         </is>
       </c>
-      <c r="H44" s="2" t="inlineStr">
+      <c r="H45" s="2" t="inlineStr">
         <is>
           <t>Application approval handling unchanged: status, Registration Document step, hardcopy resubmission
 EAINT-11763 regression (old R4). 'As before' needs that ticket's SRD/test sheet as the reference (Q-14). The checklist still lists RHB Offer Letter / Direct Debit / BoD Reso — out of scope here, note only.</t>
         </is>
       </c>
-      <c r="I44" s="2" t="inlineStr">
+      <c r="I45" s="2" t="inlineStr">
         <is>
           <t>12341_CH1</t>
         </is>
       </c>
-      <c r="J44" s="2" t="inlineStr">
+      <c r="J45" s="2" t="inlineStr">
         <is>
           <t>REQ-001 ('existing Application approval handling shall remain unchanged')</t>
         </is>
       </c>
-      <c r="K44" s="2" t="inlineStr">
+      <c r="K45" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="L44" s="2" t="inlineStr">
+      <c r="L45" s="2" t="inlineStr">
         <is>
           <t>Regression</t>
         </is>
       </c>
-      <c r="M44" s="2" t="inlineStr"/>
-      <c r="N44" s="2" t="inlineStr">
+      <c r="M45" s="2" t="inlineStr"/>
+      <c r="N45" s="2" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="O44" s="2" t="inlineStr"/>
+      <c r="O45" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="16">
@@ -2745,20 +2819,20 @@
     <mergeCell ref="B8:O8"/>
     <mergeCell ref="A20:O20"/>
     <mergeCell ref="B4:O4"/>
-    <mergeCell ref="A26:O26"/>
     <mergeCell ref="B6:O6"/>
     <mergeCell ref="B2:O2"/>
     <mergeCell ref="A14:O14"/>
+    <mergeCell ref="A33:O33"/>
     <mergeCell ref="B7:O7"/>
     <mergeCell ref="B10:O10"/>
     <mergeCell ref="B11:O11"/>
     <mergeCell ref="B3:O3"/>
     <mergeCell ref="B5:O5"/>
-    <mergeCell ref="A32:O32"/>
-    <mergeCell ref="A39:O39"/>
+    <mergeCell ref="A27:O27"/>
+    <mergeCell ref="A40:O40"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="N14:N44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="N14:N45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not Run,Pass,Fail,Blocked,N/A"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2805,7 +2879,7 @@
         </is>
       </c>
       <c r="B4" s="2">
-        <f>COUNTIF('EAINT-12341'!$A$14:$A$44,"12341_TS*")</f>
+        <f>COUNTIF('EAINT-12341'!$A$14:$A$45,"12341_TS*")</f>
         <v/>
       </c>
     </row>
@@ -2816,7 +2890,7 @@
         </is>
       </c>
       <c r="B5" s="2">
-        <f>COUNTIF('EAINT-12341'!$N$14:$N$44,"Not Run")</f>
+        <f>COUNTIF('EAINT-12341'!$N$14:$N$45,"Not Run")</f>
         <v/>
       </c>
     </row>
@@ -2827,7 +2901,7 @@
         </is>
       </c>
       <c r="B6" s="2">
-        <f>COUNTIF('EAINT-12341'!$N$14:$N$44,"Pass")</f>
+        <f>COUNTIF('EAINT-12341'!$N$14:$N$45,"Pass")</f>
         <v/>
       </c>
     </row>
@@ -2838,7 +2912,7 @@
         </is>
       </c>
       <c r="B7" s="2">
-        <f>COUNTIF('EAINT-12341'!$N$14:$N$44,"Fail")</f>
+        <f>COUNTIF('EAINT-12341'!$N$14:$N$45,"Fail")</f>
         <v/>
       </c>
     </row>
@@ -2849,7 +2923,7 @@
         </is>
       </c>
       <c r="B8" s="2">
-        <f>COUNTIF('EAINT-12341'!$N$14:$N$44,"Blocked")</f>
+        <f>COUNTIF('EAINT-12341'!$N$14:$N$45,"Blocked")</f>
         <v/>
       </c>
     </row>
@@ -2860,7 +2934,7 @@
         </is>
       </c>
       <c r="B9" s="2">
-        <f>COUNTIF('EAINT-12341'!$N$14:$N$44,"N/A")</f>
+        <f>COUNTIF('EAINT-12341'!$N$14:$N$45,"N/A")</f>
         <v/>
       </c>
     </row>
@@ -2871,7 +2945,7 @@
         </is>
       </c>
       <c r="B10" s="2">
-        <f>COUNTIF('EAINT-12341'!$K$14:$K$44,"High")</f>
+        <f>COUNTIF('EAINT-12341'!$K$14:$K$45,"High")</f>
         <v/>
       </c>
     </row>
@@ -2882,7 +2956,7 @@
         </is>
       </c>
       <c r="B11" s="2">
-        <f>COUNTIF('EAINT-12341'!$K$14:$K$44,"Medium")</f>
+        <f>COUNTIF('EAINT-12341'!$K$14:$K$45,"Medium")</f>
         <v/>
       </c>
     </row>
@@ -2893,7 +2967,7 @@
         </is>
       </c>
       <c r="B12" s="2">
-        <f>COUNTIF('EAINT-12341'!$K$14:$K$44,"Low")</f>
+        <f>COUNTIF('EAINT-12341'!$K$14:$K$45,"Low")</f>
         <v/>
       </c>
     </row>
@@ -3221,7 +3295,7 @@
         </is>
       </c>
       <c r="F4" s="2">
-        <f>COUNTIF('EAINT-12341'!$J$14:$J$44,"*REQ-001*")</f>
+        <f>COUNTIF('EAINT-12341'!$J$14:$J$45,"*REQ-001*")</f>
         <v/>
       </c>
     </row>
@@ -3252,7 +3326,7 @@
         </is>
       </c>
       <c r="F5" s="2">
-        <f>COUNTIF('EAINT-12341'!$J$14:$J$44,"*REQ-002*")</f>
+        <f>COUNTIF('EAINT-12341'!$J$14:$J$45,"*REQ-002*")</f>
         <v/>
       </c>
     </row>
@@ -3283,7 +3357,7 @@
         </is>
       </c>
       <c r="F6" s="2">
-        <f>COUNTIF('EAINT-12341'!$J$14:$J$44,"*REQ-003*")</f>
+        <f>COUNTIF('EAINT-12341'!$J$14:$J$45,"*REQ-003*")</f>
         <v/>
       </c>
     </row>
@@ -3314,7 +3388,7 @@
         </is>
       </c>
       <c r="F7" s="2">
-        <f>COUNTIF('EAINT-12341'!$J$14:$J$44,"*REQ-004*")</f>
+        <f>COUNTIF('EAINT-12341'!$J$14:$J$45,"*REQ-004*")</f>
         <v/>
       </c>
     </row>
@@ -3341,11 +3415,11 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>12341_TS02, 12341_TS03, 12341_TS04, 12341_TS06, 12341_TS07, 12341_TS08, 12341_TS09, 12341_TS10, 12341_TS21</t>
+          <t>12341_TS02, 12341_TS03, 12341_TS04, 12341_TS06, 12341_TS07, 12341_TS08, 12341_TS08A, 12341_TS09, 12341_TS10, 12341_TS21</t>
         </is>
       </c>
       <c r="F8" s="2">
-        <f>COUNTIF('EAINT-12341'!$J$14:$J$44,"*REQ-005*")</f>
+        <f>COUNTIF('EAINT-12341'!$J$14:$J$45,"*REQ-005*")</f>
         <v/>
       </c>
     </row>
@@ -3376,7 +3450,7 @@
         </is>
       </c>
       <c r="F9" s="2">
-        <f>COUNTIF('EAINT-12341'!$J$14:$J$44,"*REQ-006*")</f>
+        <f>COUNTIF('EAINT-12341'!$J$14:$J$45,"*REQ-006*")</f>
         <v/>
       </c>
     </row>
@@ -3407,7 +3481,7 @@
         </is>
       </c>
       <c r="F10" s="2">
-        <f>COUNTIF('EAINT-12341'!$J$14:$J$44,"*REQ-007*")</f>
+        <f>COUNTIF('EAINT-12341'!$J$14:$J$45,"*REQ-007*")</f>
         <v/>
       </c>
     </row>
@@ -3438,7 +3512,7 @@
         </is>
       </c>
       <c r="F11" s="2">
-        <f>COUNTIF('EAINT-12341'!$J$14:$J$44,"*REQ-008*")</f>
+        <f>COUNTIF('EAINT-12341'!$J$14:$J$45,"*REQ-008*")</f>
         <v/>
       </c>
     </row>
@@ -3469,7 +3543,7 @@
         </is>
       </c>
       <c r="F12" s="2">
-        <f>COUNTIF('EAINT-12341'!$J$14:$J$44,"*REQ-009*")</f>
+        <f>COUNTIF('EAINT-12341'!$J$14:$J$45,"*REQ-009*")</f>
         <v/>
       </c>
     </row>
@@ -3484,7 +3558,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M13"/>
+  <dimension ref="A1:M15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3720,17 +3794,17 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>12341_CH4</t>
+          <t>12341_CH8</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>LLP</t>
+          <t>Sdn Bhd / Bhd</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>4 partners</t>
+          <t>4 directors</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -3745,17 +3819,17 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>LLP business type: same template; Appointment Letter renders an LLP registration number.</t>
+          <t>Sdn Bhd normal case (REQ-005 Example 1), added at the QA's request so Sdn Bhd / Bhd is covered without a foreign director too.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>New PASS LLP company (TIN prefix PT). eSim seed: 4 PT. (Only 1 LLP was usable on the 23.09 sheet.)</t>
+          <t>New PASS ROC company (TIN prefix C). eSim: 4 DIRECTOR, all 12-digit IC.</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>12341_TS09, 12341_TS15, 12341_TS19</t>
+          <t>12341_TS08A, 12341_TS15, 12341_TS19</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr"/>
@@ -3767,17 +3841,17 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>12341_CH5</t>
+          <t>12341_CH4</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Business Trading (Sabah) or (Sarawak)</t>
+          <t>LLP</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>2 directors (typed)</t>
+          <t>4 partners</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -3792,17 +3866,17 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Non-SSM business type: 'the same email is sent to every UCD' (SRD §2.2.2). Appointment Letter BRN fields TBC (Q-09).</t>
+          <t>LLP business type: same template; Appointment Letter renders an LLP registration number.</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Unique trading licence number + licence file (pdf/png/jpg ≤5MB). TIN to use: Q-20. No eSim seed.</t>
+          <t>New PASS LLP company (TIN prefix PT). eSim seed: 4 PT. (Only 1 LLP was usable on the 23.09 sheet.)</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>12341_TS10, 12341_TS15, 12341_TS20</t>
+          <t>12341_TS09, 12341_TS15, 12341_TS19</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr"/>
@@ -3814,17 +3888,17 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>12341_CH6</t>
+          <t>12341_CH5</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Sole Proprietorship / Partnership</t>
+          <t>Business Trading (Sabah)</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>4 business owners</t>
+          <t>2 directors (typed)</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -3834,22 +3908,22 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Application Submitted (then manual Revert to UCD)</t>
+          <t>Application Approved</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Negative trigger: no new email at Submitted or on Revert to UCD (REQ-001).</t>
+          <t>Non-SSM business type: 'the same email is sent to every UCD' (SRD §2.2.2). Appointment Letter BRN fields TBC (Q-09).</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>New PASS ROB company. eSim seed: 4 CURRENT_OWNER.</t>
+          <t>Unique trading licence number (robot generates) + licence file (sample provided). TIN to use: Q-20. No eSim setup.</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>12341_TS25</t>
+          <t>12341_TS10, 12341_TS15, 12341_TS20</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr"/>
@@ -3858,22 +3932,116 @@
       <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="2" t="inlineStr"/>
     </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>12341_CH7</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Business Trading (Sarawak)</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>2 directors (typed)</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>All Malaysian</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Application Approved</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Second non-SSM business type (Sarawak) — every business type on the Pre-Application form is covered once.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Same as CH5, region Sarawak. TIN to use: Q-20. No eSim setup.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>12341_TS10, 12341_TS15, 12341_TS20</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr"/>
+    </row>
     <row r="11">
-      <c r="A11" s="10" t="inlineStr">
-        <is>
-          <t>Fill columns I–M after each run from the run log's READY FOR MANUAL EMAIL CHECK block.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="10" t="inlineStr">
-        <is>
-          <t>Spent companies from the v1.1 attempts (do not reuse): IP0581553-U (E2E1), 003270488-X (E2E2), 1267419-A (E2E6). See company-ledger.json.</t>
-        </is>
-      </c>
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>12341_CH6</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Sole Proprietorship / Partnership</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>4 business owners</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>All Malaysian</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Application Submitted (then manual Revert to UCD)</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Negative trigger: no new email at Submitted or on Revert to UCD (REQ-001).</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>New PASS ROB company. eSim seed: 4 CURRENT_OWNER.</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>12341_TS25</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr"/>
+      <c r="M11" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Fill columns I–M after each run from the run log's READY FOR MANUAL EMAIL CHECK block.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>Spent companies from the v1.1 attempts (do not reuse): IP0581553-U (E2E1), 003270488-X (E2E2), 1267419-A (E2E6). See company-ledger.json.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>Admin In Charge and Director in Charge use DIFFERENT name / mobile / email on purpose (Q-04): the emails then show which source the system uses.</t>
         </is>
@@ -5101,7 +5269,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Test data: please share a fresh company-details-checker sheet (PASS rows) — needed: 3 ROB (TIN D), 1 ROC (TIN C), 1 LLP (TIN PT). For Business Trading (CH5): which TIN may be used (Application step 1 makes TIN mandatory)?</t>
+          <t>Test data: please share a fresh company-details-checker sheet (PASS rows) — needed: 3 ROB (TIN D), 2 ROC (TIN C), 1 LLP (TIN PT). For Business Trading (CH5 Sabah, CH7 Sarawak): which TINs may be used (Application step 1 makes TIN mandatory)?</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -5111,7 +5279,7 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>CH1–CH6</t>
+          <t>CH1–CH8</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
@@ -5464,7 +5632,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Replaced by TS10 (template now confirmed) + TS20 (letter BRN TBC).</t>
+          <t>Replaced by TS10 (template now confirmed, Sabah CH5 + Sarawak CH7) + TS20 (letter BRN TBC).</t>
         </is>
       </c>
     </row>

</xml_diff>